<commit_message>
Dashboard and reports: sales, gross profit, expenses, net profit; free price edits down to the minimum
- Dashboard (with profit access) shows, in order: المبيعات (الإيرادات),
  إجمالي الربح (sales − purchase cost), المصروفات (operating expenses incl.
  salaries/repairs + stock losses), صافي الربح (gross profit − expenses).
  Reports and the Excel export use the same names and formulas.
- Any seller may change a line's price; nobody (administrator included) may go
  under the product's minimum sale price. A changed price is no longer counted
  as a discount; only line/invoice discounts need the permission and the limit.
- POS search results and product cards show the minimum sale price.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Qwader-Test-Cases.xlsx
+++ b/docs/Qwader-Test-Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Qwader\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EE0F021-0AE3-402E-8E6E-B2BA44E31193}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5817B7A6-8AD1-46F5-B983-3E05051B4FAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2055" uniqueCount="980">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2055" uniqueCount="981">
   <si>
     <t>رقم الحالة</t>
   </si>
@@ -1318,19 +1318,24 @@
     <t>POS-05</t>
   </si>
   <si>
-    <t>البيع بأقل من الحد الأدنى</t>
-  </si>
-  <si>
-    <t>منتج حده الأدنى 85</t>
-  </si>
-  <si>
-    <t>1. غيّر السعر إلى 80 واعتمد</t>
-  </si>
-  <si>
-    <t>رسالة رفض لموظف المبيعات</t>
-  </si>
-  <si>
-    <t>رُفض: الخصم (33.3%) يتجاوز الحد المسموح (10%)</t>
+    <t>تعديل السعر حتى أقل سعر بيع فقط</t>
+  </si>
+  <si>
+    <t>منتج سعره 100 وأقل سعر بيع 70</t>
+  </si>
+  <si>
+    <t>1. اضغط على المنتج في الفاتورة
+2. غيّر السعر إلى 75 واحفظ
+3. غيّره إلى 69</t>
+  </si>
+  <si>
+    <t>75 مقبول (تعديل السعر ليس خصمًا)؛ 69 مرفوض «لا يمكن البيع بأقل من أقل سعر بيع» — حتى لمدير النظام</t>
+  </si>
+  <si>
+    <t>Any_seller_may_change_the_price_down_to_the_minimum_and_nobody_below_it</t>
+  </si>
+  <si>
+    <t>موظف مبيعات عدّل السعر إلى أقل سعر بيع (70 من 85.5) وباع؛ وتحته بـ 1 ظهرت «لا يمكن البيع بأقل من أقل سعر بيع (70.00 ₪)»</t>
   </si>
   <si>
     <t>POS-06</t>
@@ -2131,16 +2136,16 @@
     <t>1. افتح لوحة التحكم</t>
   </si>
   <si>
-    <t>مبيعات اليوم، عدد الفواتير، المبالغ المستلمة، ربح اليوم تطابق الفواتير</t>
-  </si>
-  <si>
-    <t>مبيعات اليوم 1,760.00 في 12 فاتورة تطابق التقرير</t>
+    <t>بالترتيب: المبيعات (الإيرادات)، إجمالي الربح، المصروفات، صافي الربح — وتطابق التقارير</t>
+  </si>
+  <si>
+    <t>171 مبيعات − 133 سعر شراء = 38 إجمالي ربح؛ 50 راتب؛ صافي الربح −12 — بالترتيب المطلوب</t>
   </si>
   <si>
     <t>RPT-02</t>
   </si>
   <si>
-    <t>تقرير الإيرادات والمصروفات والربح</t>
+    <t>تقرير المبيعات وإجمالي الربح والمصروفات وصافي الربح</t>
   </si>
   <si>
     <t>بيع + مرتجع + تالف + مصروف</t>
@@ -2149,7 +2154,7 @@
     <t>1. التقارير ← اليوم</t>
   </si>
   <si>
-    <t>الإيرادات = المبيعات − الخصومات − المرتجعات؛ المصروفات = ثمن البضاعة المباعة + التالف + المصاريف؛ الربح = الإيرادات − المصروفات</t>
+    <t>المبيعات (الإيرادات) = المبيعات − الخصومات − المرتجعات؛ إجمالي الربح = المبيعات − سعر الشراء؛ المصروفات = رواتب وأعطال ومصاريف تشغيلية + التالف؛ صافي الربح = إجمالي الربح − المصروفات</t>
   </si>
   <si>
     <t>Profit_and_loss_follows_the_accounting_rules</t>
@@ -2270,7 +2275,7 @@
     <t>الزيادة تظهر منفصلة («زيادة جرد لا تُحسب ربحًا») ولا يتغير الربح</t>
   </si>
   <si>
-    <t>Stock_found_or_counted_over_is_not_profit_and_profit_is_revenue_minus_expenses</t>
+    <t>Stock_found_or_counted_over_is_not_profit_and_net_profit_is_gross_profit_minus_expenses</t>
   </si>
   <si>
     <t>خطأ اكتُشف وأُصلح: زيادة الجرد كانت تُحسب ربحًا. الآن تظهر منفصلة ولا تدخل في الربح.</t>
@@ -3590,55 +3595,55 @@
   <sheetData>
     <row r="1" spans="1:2" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>912</v>
+        <v>913</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>915</v>
+        <v>916</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>916</v>
+        <v>917</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>917</v>
+        <v>918</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>919</v>
+        <v>920</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>921</v>
+        <v>922</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.25">
@@ -3646,196 +3651,196 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>924</v>
+        <v>925</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>926</v>
+        <v>927</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>927</v>
+        <v>928</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>928</v>
+        <v>929</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>929</v>
+        <v>930</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>930</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>931</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>931</v>
+        <v>932</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>932</v>
+        <v>933</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>934</v>
+        <v>935</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>935</v>
+        <v>936</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>937</v>
+        <v>938</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>938</v>
+        <v>939</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>940</v>
+        <v>941</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>941</v>
+        <v>942</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
-        <v>942</v>
+        <v>943</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>943</v>
+        <v>944</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>944</v>
+        <v>945</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
-        <v>946</v>
+        <v>947</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>948</v>
+        <v>949</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
-        <v>954</v>
+        <v>955</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
     </row>
   </sheetData>
@@ -3905,7 +3910,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>14</v>
       </c>
@@ -3949,7 +3954,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>27</v>
       </c>
@@ -3993,7 +3998,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>33</v>
       </c>
@@ -4037,7 +4042,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>41</v>
       </c>
@@ -4081,7 +4086,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>47</v>
       </c>
@@ -4125,7 +4130,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>53</v>
       </c>
@@ -4169,7 +4174,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>59</v>
       </c>
@@ -4213,7 +4218,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>65</v>
       </c>
@@ -4257,7 +4262,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
         <v>70</v>
       </c>
@@ -4301,7 +4306,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>76</v>
       </c>
@@ -4345,7 +4350,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
         <v>82</v>
       </c>
@@ -4389,7 +4394,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>88</v>
       </c>
@@ -4433,7 +4438,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
         <v>94</v>
       </c>
@@ -4477,7 +4482,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>100</v>
       </c>
@@ -4521,7 +4526,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
         <v>105</v>
       </c>
@@ -4565,7 +4570,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
         <v>111</v>
       </c>
@@ -4609,7 +4614,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
         <v>117</v>
       </c>
@@ -4653,7 +4658,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
         <v>123</v>
       </c>
@@ -4697,7 +4702,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
         <v>128</v>
       </c>
@@ -4741,7 +4746,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
         <v>133</v>
       </c>
@@ -4785,7 +4790,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
         <v>138</v>
       </c>
@@ -4829,7 +4834,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
         <v>144</v>
       </c>
@@ -4873,7 +4878,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
         <v>151</v>
       </c>
@@ -4917,7 +4922,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
         <v>158</v>
       </c>
@@ -4961,7 +4966,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
         <v>164</v>
       </c>
@@ -5005,7 +5010,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
         <v>169</v>
       </c>
@@ -5049,7 +5054,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
         <v>175</v>
       </c>
@@ -5093,7 +5098,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
         <v>180</v>
       </c>
@@ -5137,7 +5142,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
         <v>187</v>
       </c>
@@ -5181,7 +5186,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
         <v>193</v>
       </c>
@@ -5225,7 +5230,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
         <v>200</v>
       </c>
@@ -5269,7 +5274,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
         <v>205</v>
       </c>
@@ -5313,7 +5318,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
         <v>210</v>
       </c>
@@ -5357,7 +5362,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
         <v>215</v>
       </c>
@@ -5401,7 +5406,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
         <v>223</v>
       </c>
@@ -5445,7 +5450,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
         <v>228</v>
       </c>
@@ -5489,7 +5494,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="38" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
         <v>235</v>
       </c>
@@ -5533,7 +5538,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="39" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
         <v>242</v>
       </c>
@@ -5577,7 +5582,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="40" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
         <v>249</v>
       </c>
@@ -5621,7 +5626,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="41" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
         <v>256</v>
       </c>
@@ -5665,7 +5670,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
         <v>262</v>
       </c>
@@ -5709,7 +5714,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="43" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
         <v>269</v>
       </c>
@@ -5753,7 +5758,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="44" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
         <v>276</v>
       </c>
@@ -5797,7 +5802,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="45" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
         <v>282</v>
       </c>
@@ -5841,7 +5846,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="46" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
         <v>286</v>
       </c>
@@ -5885,7 +5890,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
         <v>292</v>
       </c>
@@ -5929,7 +5934,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="48" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
         <v>299</v>
       </c>
@@ -5973,7 +5978,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="49" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
         <v>305</v>
       </c>
@@ -6017,7 +6022,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="50" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
         <v>311</v>
       </c>
@@ -6061,7 +6066,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="51" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
         <v>318</v>
       </c>
@@ -6105,7 +6110,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="52" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
         <v>325</v>
       </c>
@@ -6149,7 +6154,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="53" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
         <v>332</v>
       </c>
@@ -6193,7 +6198,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="54" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
         <v>337</v>
       </c>
@@ -6237,7 +6242,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="55" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
         <v>343</v>
       </c>
@@ -6281,7 +6286,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="56" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
         <v>348</v>
       </c>
@@ -6325,7 +6330,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
         <v>355</v>
       </c>
@@ -6369,7 +6374,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
         <v>362</v>
       </c>
@@ -6413,7 +6418,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="59" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
         <v>368</v>
       </c>
@@ -6457,7 +6462,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="60" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
         <v>375</v>
       </c>
@@ -6501,7 +6506,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="61" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
         <v>381</v>
       </c>
@@ -6545,7 +6550,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
         <v>389</v>
       </c>
@@ -6589,7 +6594,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
         <v>396</v>
       </c>
@@ -6633,7 +6638,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="64" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
         <v>402</v>
       </c>
@@ -6677,7 +6682,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="65" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
         <v>406</v>
       </c>
@@ -6721,7 +6726,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="66" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
         <v>412</v>
       </c>
@@ -6750,13 +6755,13 @@
         <v>22</v>
       </c>
       <c r="J66" s="12" t="s">
-        <v>149</v>
+        <v>417</v>
       </c>
       <c r="K66" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L66" s="14" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="M66" s="13" t="s">
         <v>26</v>
@@ -6765,15 +6770,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="67" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B67" s="11" t="s">
         <v>390</v>
       </c>
       <c r="C67" s="11" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D67" s="10" t="s">
         <v>119</v>
@@ -6782,10 +6787,10 @@
         <v>29</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="G67" s="11" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="H67" s="10" t="s">
         <v>38</v>
@@ -6794,13 +6799,13 @@
         <v>22</v>
       </c>
       <c r="J67" s="12" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="K67" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L67" s="14" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="M67" s="13" t="s">
         <v>26</v>
@@ -6809,15 +6814,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="68" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B68" s="11" t="s">
         <v>390</v>
       </c>
       <c r="C68" s="11" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D68" s="10" t="s">
         <v>119</v>
@@ -6826,10 +6831,10 @@
         <v>29</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="G68" s="11" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="H68" s="10" t="s">
         <v>21</v>
@@ -6838,13 +6843,13 @@
         <v>22</v>
       </c>
       <c r="J68" s="12" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K68" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L68" s="14" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="M68" s="13" t="s">
         <v>26</v>
@@ -6853,15 +6858,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="69" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B69" s="11" t="s">
         <v>390</v>
       </c>
       <c r="C69" s="11" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="D69" s="10" t="s">
         <v>119</v>
@@ -6870,10 +6875,10 @@
         <v>29</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="G69" s="11" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="H69" s="10" t="s">
         <v>21</v>
@@ -6882,13 +6887,13 @@
         <v>22</v>
       </c>
       <c r="J69" s="12" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K69" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L69" s="14" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="M69" s="13" t="s">
         <v>26</v>
@@ -6897,27 +6902,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="70" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>390</v>
       </c>
       <c r="C70" s="11" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="D70" s="10" t="s">
         <v>119</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="G70" s="11" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="H70" s="10" t="s">
         <v>38</v>
@@ -6926,13 +6931,13 @@
         <v>22</v>
       </c>
       <c r="J70" s="12" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K70" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L70" s="14" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="M70" s="13" t="s">
         <v>26</v>
@@ -6941,15 +6946,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="71" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B71" s="11" t="s">
         <v>390</v>
       </c>
       <c r="C71" s="11" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D71" s="10" t="s">
         <v>119</v>
@@ -6958,10 +6963,10 @@
         <v>29</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G71" s="11" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="H71" s="10" t="s">
         <v>21</v>
@@ -6976,7 +6981,7 @@
         <v>24</v>
       </c>
       <c r="L71" s="14" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="M71" s="13" t="s">
         <v>26</v>
@@ -6985,15 +6990,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="72" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B72" s="11" t="s">
         <v>390</v>
       </c>
       <c r="C72" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D72" s="10" t="s">
         <v>119</v>
@@ -7002,10 +7007,10 @@
         <v>153</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="G72" s="11" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="H72" s="10" t="s">
         <v>21</v>
@@ -7014,13 +7019,13 @@
         <v>22</v>
       </c>
       <c r="J72" s="12" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="K72" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L72" s="14" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="M72" s="13" t="s">
         <v>26</v>
@@ -7029,15 +7034,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="73" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B73" s="11" t="s">
         <v>390</v>
       </c>
       <c r="C73" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D73" s="10" t="s">
         <v>119</v>
@@ -7046,10 +7051,10 @@
         <v>320</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="G73" s="11" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="H73" s="10" t="s">
         <v>21</v>
@@ -7058,13 +7063,13 @@
         <v>22</v>
       </c>
       <c r="J73" s="12" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="K73" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L73" s="14" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="M73" s="13" t="s">
         <v>26</v>
@@ -7073,27 +7078,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="74" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B74" s="11" t="s">
         <v>390</v>
       </c>
       <c r="C74" s="11" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D74" s="10" t="s">
         <v>119</v>
       </c>
       <c r="E74" s="11" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="G74" s="11" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="H74" s="10" t="s">
         <v>21</v>
@@ -7102,13 +7107,13 @@
         <v>22</v>
       </c>
       <c r="J74" s="12" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K74" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L74" s="14" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="M74" s="13" t="s">
         <v>26</v>
@@ -7117,27 +7122,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="75" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="10" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B75" s="11" t="s">
         <v>390</v>
       </c>
       <c r="C75" s="11" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="D75" s="10" t="s">
         <v>119</v>
       </c>
       <c r="E75" s="11" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="F75" s="11" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="G75" s="11" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="H75" s="10" t="s">
         <v>38</v>
@@ -7161,27 +7166,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="76" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="10" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B76" s="11" t="s">
         <v>390</v>
       </c>
       <c r="C76" s="11" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="D76" s="10" t="s">
         <v>119</v>
       </c>
       <c r="E76" s="11" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="F76" s="11" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="G76" s="11" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="H76" s="10" t="s">
         <v>38</v>
@@ -7196,7 +7201,7 @@
         <v>24</v>
       </c>
       <c r="L76" s="14" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="M76" s="13" t="s">
         <v>26</v>
@@ -7205,27 +7210,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="77" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="10" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B77" s="11" t="s">
         <v>390</v>
       </c>
       <c r="C77" s="11" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="D77" s="10" t="s">
         <v>171</v>
       </c>
       <c r="E77" s="11" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="F77" s="11" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="G77" s="11" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="H77" s="10" t="s">
         <v>38</v>
@@ -7249,27 +7254,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="78" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="10" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B78" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C78" s="11" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="D78" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E78" s="11" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F78" s="11" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="G78" s="11" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="H78" s="10" t="s">
         <v>38</v>
@@ -7293,27 +7298,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="79" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="10" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B79" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C79" s="11" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="D79" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E79" s="11" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="F79" s="11" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="G79" s="11" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="H79" s="10" t="s">
         <v>38</v>
@@ -7337,27 +7342,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="80" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="10" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B80" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C80" s="11" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="D80" s="10" t="s">
         <v>383</v>
       </c>
       <c r="E80" s="11" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="F80" s="11" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="G80" s="11" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="H80" s="10" t="s">
         <v>21</v>
@@ -7372,7 +7377,7 @@
         <v>24</v>
       </c>
       <c r="L80" s="14" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="M80" s="13" t="s">
         <v>26</v>
@@ -7381,27 +7386,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="81" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="10" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="B81" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C81" s="11" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D81" s="10" t="s">
         <v>119</v>
       </c>
       <c r="E81" s="11" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="F81" s="11" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="G81" s="11" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="H81" s="10" t="s">
         <v>21</v>
@@ -7410,7 +7415,7 @@
         <v>22</v>
       </c>
       <c r="J81" s="12" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="K81" s="13" t="s">
         <v>24</v>
@@ -7425,27 +7430,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="82" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="10" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B82" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C82" s="11" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="D82" s="10" t="s">
         <v>119</v>
       </c>
       <c r="E82" s="11" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="F82" s="11" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="G82" s="11" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="H82" s="10" t="s">
         <v>21</v>
@@ -7454,13 +7459,13 @@
         <v>22</v>
       </c>
       <c r="J82" s="12" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="K82" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L82" s="14" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="M82" s="13" t="s">
         <v>26</v>
@@ -7469,27 +7474,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="83" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="10" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B83" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C83" s="11" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="D83" s="10" t="s">
         <v>119</v>
       </c>
       <c r="E83" s="11" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F83" s="11" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="G83" s="11" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="H83" s="10" t="s">
         <v>38</v>
@@ -7498,13 +7503,13 @@
         <v>22</v>
       </c>
       <c r="J83" s="12" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="K83" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L83" s="14" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="M83" s="13" t="s">
         <v>26</v>
@@ -7513,24 +7518,24 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="84" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="10" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B84" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C84" s="11" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="D84" s="10" t="s">
         <v>119</v>
       </c>
       <c r="E84" s="11" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="F84" s="11" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="G84" s="11" t="s">
         <v>260</v>
@@ -7542,13 +7547,13 @@
         <v>22</v>
       </c>
       <c r="J84" s="12" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="K84" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L84" s="14" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="M84" s="13" t="s">
         <v>26</v>
@@ -7557,27 +7562,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="85" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="10" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B85" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C85" s="11" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="D85" s="10" t="s">
         <v>119</v>
       </c>
       <c r="E85" s="11" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="F85" s="11" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="G85" s="11" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="H85" s="10" t="s">
         <v>21</v>
@@ -7586,13 +7591,13 @@
         <v>22</v>
       </c>
       <c r="J85" s="12" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="K85" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L85" s="14" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="M85" s="13" t="s">
         <v>26</v>
@@ -7601,27 +7606,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="86" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="10" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B86" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C86" s="11" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="D86" s="10" t="s">
         <v>171</v>
       </c>
       <c r="E86" s="11" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="F86" s="11" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="G86" s="11" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="H86" s="10" t="s">
         <v>21</v>
@@ -7630,7 +7635,7 @@
         <v>22</v>
       </c>
       <c r="J86" s="12" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="K86" s="13" t="s">
         <v>24</v>
@@ -7645,24 +7650,24 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="87" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="10" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B87" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C87" s="11" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D87" s="10" t="s">
         <v>171</v>
       </c>
       <c r="E87" s="11" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="F87" s="11" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="G87" s="11" t="s">
         <v>260</v>
@@ -7674,13 +7679,13 @@
         <v>22</v>
       </c>
       <c r="J87" s="12" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="K87" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L87" s="14" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="M87" s="13" t="s">
         <v>26</v>
@@ -7689,27 +7694,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="88" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="10" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B88" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C88" s="11" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="D88" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E88" s="11" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F88" s="11" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="G88" s="11" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="H88" s="10" t="s">
         <v>80</v>
@@ -7724,7 +7729,7 @@
         <v>24</v>
       </c>
       <c r="L88" s="14" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="M88" s="13" t="s">
         <v>26</v>
@@ -7733,15 +7738,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="89" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="10" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B89" s="11" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C89" s="11" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="D89" s="10" t="s">
         <v>119</v>
@@ -7750,10 +7755,10 @@
         <v>29</v>
       </c>
       <c r="F89" s="11" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="G89" s="11" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="H89" s="10" t="s">
         <v>38</v>
@@ -7777,27 +7782,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="90" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="10" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B90" s="11" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C90" s="11" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="D90" s="10" t="s">
         <v>383</v>
       </c>
       <c r="E90" s="11" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="F90" s="11" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="G90" s="11" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="H90" s="10" t="s">
         <v>21</v>
@@ -7806,13 +7811,13 @@
         <v>22</v>
       </c>
       <c r="J90" s="12" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="K90" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L90" s="14" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="M90" s="13" t="s">
         <v>26</v>
@@ -7821,27 +7826,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="91" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="10" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="B91" s="11" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C91" s="11" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="D91" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E91" s="11" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="F91" s="11" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="G91" s="11" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="H91" s="10" t="s">
         <v>38</v>
@@ -7865,27 +7870,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="92" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="10" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="B92" s="11" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C92" s="11" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D92" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E92" s="11" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="F92" s="11" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="G92" s="11" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="H92" s="10" t="s">
         <v>80</v>
@@ -7900,7 +7905,7 @@
         <v>24</v>
       </c>
       <c r="L92" s="14" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="M92" s="13" t="s">
         <v>26</v>
@@ -7909,27 +7914,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="93" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="10" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="B93" s="11" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C93" s="11" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="D93" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E93" s="11" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="F93" s="11" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="G93" s="11" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="H93" s="10" t="s">
         <v>38</v>
@@ -7953,15 +7958,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="94" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="10" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="B94" s="11" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="C94" s="11" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="D94" s="10" t="s">
         <v>119</v>
@@ -7970,10 +7975,10 @@
         <v>29</v>
       </c>
       <c r="F94" s="11" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="G94" s="11" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="H94" s="10" t="s">
         <v>21</v>
@@ -7982,13 +7987,13 @@
         <v>22</v>
       </c>
       <c r="J94" s="12" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="K94" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L94" s="14" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="M94" s="13" t="s">
         <v>26</v>
@@ -7997,27 +8002,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="95" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="10" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B95" s="11" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="C95" s="11" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="D95" s="10" t="s">
         <v>383</v>
       </c>
       <c r="E95" s="11" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="F95" s="11" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="G95" s="11" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="H95" s="10" t="s">
         <v>21</v>
@@ -8026,13 +8031,13 @@
         <v>22</v>
       </c>
       <c r="J95" s="12" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="K95" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L95" s="14" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="M95" s="13" t="s">
         <v>26</v>
@@ -8041,27 +8046,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="96" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="10" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B96" s="11" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="C96" s="11" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="D96" s="10" t="s">
         <v>383</v>
       </c>
       <c r="E96" s="11" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="F96" s="11" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="G96" s="11" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="H96" s="10" t="s">
         <v>21</v>
@@ -8070,7 +8075,7 @@
         <v>22</v>
       </c>
       <c r="J96" s="12" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="K96" s="13" t="s">
         <v>24</v>
@@ -8085,27 +8090,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="97" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:14" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="10" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B97" s="11" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="C97" s="11" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D97" s="10" t="s">
         <v>119</v>
       </c>
       <c r="E97" s="11" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="F97" s="11" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="G97" s="11" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="H97" s="10" t="s">
         <v>21</v>
@@ -8114,13 +8119,13 @@
         <v>22</v>
       </c>
       <c r="J97" s="12" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="K97" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L97" s="14" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="M97" s="13" t="s">
         <v>26</v>
@@ -8129,27 +8134,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="98" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="10" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="B98" s="11" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="C98" s="11" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="D98" s="10" t="s">
         <v>383</v>
       </c>
       <c r="E98" s="11" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="F98" s="11" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="G98" s="11" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="H98" s="10" t="s">
         <v>38</v>
@@ -8164,7 +8169,7 @@
         <v>24</v>
       </c>
       <c r="L98" s="14" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="M98" s="13" t="s">
         <v>26</v>
@@ -8173,27 +8178,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="99" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="10" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="B99" s="11" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="C99" s="11" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="D99" s="10" t="s">
         <v>383</v>
       </c>
       <c r="E99" s="11" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="F99" s="11" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="G99" s="11" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="H99" s="10" t="s">
         <v>80</v>
@@ -8217,27 +8222,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="100" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="10" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B100" s="11" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="C100" s="11" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="D100" s="10" t="s">
         <v>85</v>
       </c>
       <c r="E100" s="11" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="F100" s="11" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="G100" s="11" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="H100" s="10" t="s">
         <v>38</v>
@@ -8246,7 +8251,7 @@
         <v>22</v>
       </c>
       <c r="J100" s="12" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="K100" s="13" t="s">
         <v>24</v>
@@ -8261,15 +8266,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="101" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="10" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="B101" s="11" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="C101" s="11" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="D101" s="10" t="s">
         <v>85</v>
@@ -8278,10 +8283,10 @@
         <v>29</v>
       </c>
       <c r="F101" s="11" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="G101" s="11" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="H101" s="10" t="s">
         <v>21</v>
@@ -8290,7 +8295,7 @@
         <v>22</v>
       </c>
       <c r="J101" s="12" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="K101" s="13" t="s">
         <v>24</v>
@@ -8305,27 +8310,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="102" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="10" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B102" s="11" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="C102" s="11" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="D102" s="10" t="s">
         <v>383</v>
       </c>
       <c r="E102" s="11" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="F102" s="11" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="G102" s="11" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="H102" s="10" t="s">
         <v>21</v>
@@ -8334,7 +8339,7 @@
         <v>22</v>
       </c>
       <c r="J102" s="12" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="K102" s="13" t="s">
         <v>24</v>
@@ -8349,27 +8354,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="103" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="10" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="B103" s="11" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="C103" s="11" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="D103" s="10" t="s">
         <v>383</v>
       </c>
       <c r="E103" s="11" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="F103" s="11" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="G103" s="11" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="H103" s="10" t="s">
         <v>21</v>
@@ -8378,13 +8383,13 @@
         <v>22</v>
       </c>
       <c r="J103" s="12" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="K103" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L103" s="14" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="M103" s="13" t="s">
         <v>26</v>
@@ -8393,27 +8398,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="104" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="10" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="B104" s="11" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="C104" s="11" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="D104" s="10" t="s">
         <v>119</v>
       </c>
       <c r="E104" s="11" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="F104" s="11" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="G104" s="11" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="H104" s="10" t="s">
         <v>38</v>
@@ -8422,13 +8427,13 @@
         <v>22</v>
       </c>
       <c r="J104" s="12" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="K104" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L104" s="14" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="M104" s="13" t="s">
         <v>26</v>
@@ -8437,27 +8442,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="105" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="10" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B105" s="11" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C105" s="11" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="D105" s="10" t="s">
         <v>383</v>
       </c>
       <c r="E105" s="11" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="F105" s="11" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="G105" s="11" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="H105" s="10" t="s">
         <v>21</v>
@@ -8466,13 +8471,13 @@
         <v>22</v>
       </c>
       <c r="J105" s="12" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="K105" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L105" s="14" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="M105" s="13" t="s">
         <v>26</v>
@@ -8481,27 +8486,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="106" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="10" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B106" s="11" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C106" s="11" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="D106" s="10" t="s">
         <v>383</v>
       </c>
       <c r="E106" s="11" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="F106" s="11" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="G106" s="11" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="H106" s="10" t="s">
         <v>21</v>
@@ -8510,7 +8515,7 @@
         <v>22</v>
       </c>
       <c r="J106" s="12" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="K106" s="13" t="s">
         <v>24</v>
@@ -8525,27 +8530,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="107" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="10" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="B107" s="11" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C107" s="11" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="D107" s="10" t="s">
         <v>383</v>
       </c>
       <c r="E107" s="11" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="F107" s="11" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="G107" s="11" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="H107" s="10" t="s">
         <v>21</v>
@@ -8554,13 +8559,13 @@
         <v>22</v>
       </c>
       <c r="J107" s="12" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K107" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L107" s="14" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="M107" s="13" t="s">
         <v>26</v>
@@ -8569,15 +8574,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="108" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="10" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="B108" s="11" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C108" s="11" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="D108" s="10" t="s">
         <v>383</v>
@@ -8586,10 +8591,10 @@
         <v>29</v>
       </c>
       <c r="F108" s="11" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="G108" s="11" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="H108" s="10" t="s">
         <v>21</v>
@@ -8598,7 +8603,7 @@
         <v>22</v>
       </c>
       <c r="J108" s="12" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="K108" s="13" t="s">
         <v>24</v>
@@ -8613,27 +8618,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="109" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="10" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B109" s="11" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C109" s="11" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="D109" s="10" t="s">
         <v>383</v>
       </c>
       <c r="E109" s="11" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F109" s="11" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="G109" s="11" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="H109" s="10" t="s">
         <v>21</v>
@@ -8642,7 +8647,7 @@
         <v>22</v>
       </c>
       <c r="J109" s="12" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="K109" s="13" t="s">
         <v>24</v>
@@ -8657,27 +8662,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="110" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="10" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B110" s="11" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C110" s="11" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="D110" s="10" t="s">
         <v>383</v>
       </c>
       <c r="E110" s="11" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="F110" s="11" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="G110" s="11" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="H110" s="10" t="s">
         <v>80</v>
@@ -8692,7 +8697,7 @@
         <v>24</v>
       </c>
       <c r="L110" s="14" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="M110" s="13" t="s">
         <v>26</v>
@@ -8701,27 +8706,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="111" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="10" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="B111" s="11" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="C111" s="11" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="D111" s="10" t="s">
         <v>85</v>
       </c>
       <c r="E111" s="11" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="F111" s="11" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="G111" s="11" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="H111" s="10" t="s">
         <v>21</v>
@@ -8736,7 +8741,7 @@
         <v>24</v>
       </c>
       <c r="L111" s="14" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="M111" s="13" t="s">
         <v>26</v>
@@ -8745,27 +8750,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="112" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="10" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="B112" s="11" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="C112" s="11" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="D112" s="10" t="s">
         <v>85</v>
       </c>
       <c r="E112" s="11" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="F112" s="11" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="G112" s="11" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="H112" s="10" t="s">
         <v>21</v>
@@ -8774,13 +8779,13 @@
         <v>22</v>
       </c>
       <c r="J112" s="12" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="K112" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L112" s="14" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="M112" s="13" t="s">
         <v>26</v>
@@ -8789,27 +8794,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="113" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="10" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B113" s="11" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="C113" s="11" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="D113" s="10" t="s">
         <v>85</v>
       </c>
       <c r="E113" s="11" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="F113" s="11" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="G113" s="11" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="H113" s="10" t="s">
         <v>38</v>
@@ -8818,13 +8823,13 @@
         <v>22</v>
       </c>
       <c r="J113" s="12" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="K113" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L113" s="14" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="M113" s="13" t="s">
         <v>26</v>
@@ -8833,15 +8838,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="114" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="10" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B114" s="11" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="C114" s="11" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="D114" s="10" t="s">
         <v>85</v>
@@ -8850,10 +8855,10 @@
         <v>29</v>
       </c>
       <c r="F114" s="11" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="G114" s="11" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="H114" s="10" t="s">
         <v>80</v>
@@ -8862,13 +8867,13 @@
         <v>22</v>
       </c>
       <c r="J114" s="12" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="K114" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L114" s="14" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="M114" s="13" t="s">
         <v>26</v>
@@ -8877,27 +8882,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="115" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="10" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B115" s="11" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="C115" s="11" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="D115" s="10" t="s">
         <v>85</v>
       </c>
       <c r="E115" s="11" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="F115" s="11" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="G115" s="11" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="H115" s="10" t="s">
         <v>38</v>
@@ -8921,15 +8926,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="116" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="10" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B116" s="11" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="C116" s="11" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="D116" s="10" t="s">
         <v>383</v>
@@ -8938,10 +8943,10 @@
         <v>29</v>
       </c>
       <c r="F116" s="11" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="G116" s="11" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="H116" s="10" t="s">
         <v>38</v>
@@ -8965,27 +8970,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="117" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="10" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B117" s="11" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="C117" s="11" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="D117" s="10" t="s">
         <v>85</v>
       </c>
       <c r="E117" s="11" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F117" s="11" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="G117" s="11" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="H117" s="10" t="s">
         <v>38</v>
@@ -8994,13 +8999,13 @@
         <v>22</v>
       </c>
       <c r="J117" s="12" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="K117" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L117" s="14" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="M117" s="13" t="s">
         <v>26</v>
@@ -9009,15 +9014,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="118" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="10" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B118" s="11" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="C118" s="11" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="D118" s="10" t="s">
         <v>119</v>
@@ -9026,10 +9031,10 @@
         <v>29</v>
       </c>
       <c r="F118" s="11" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="G118" s="11" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="H118" s="10" t="s">
         <v>21</v>
@@ -9038,7 +9043,7 @@
         <v>22</v>
       </c>
       <c r="J118" s="12" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="K118" s="13" t="s">
         <v>24</v>
@@ -9053,27 +9058,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="119" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="10" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B119" s="11" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="C119" s="11" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="D119" s="10" t="s">
         <v>85</v>
       </c>
       <c r="E119" s="11" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="F119" s="11" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="G119" s="11" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="H119" s="10" t="s">
         <v>21</v>
@@ -9082,13 +9087,13 @@
         <v>22</v>
       </c>
       <c r="J119" s="12" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="K119" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L119" s="14" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="M119" s="13" t="s">
         <v>26</v>
@@ -9097,15 +9102,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="120" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="10" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="B120" s="11" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="C120" s="11" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="D120" s="10" t="s">
         <v>17</v>
@@ -9114,10 +9119,10 @@
         <v>29</v>
       </c>
       <c r="F120" s="11" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="G120" s="11" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="H120" s="10" t="s">
         <v>38</v>
@@ -9141,27 +9146,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="121" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="10" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B121" s="11" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="C121" s="11" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="D121" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E121" s="11" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="F121" s="11" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="G121" s="11" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="H121" s="10" t="s">
         <v>38</v>
@@ -9176,7 +9181,7 @@
         <v>24</v>
       </c>
       <c r="L121" s="14" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="M121" s="13" t="s">
         <v>26</v>
@@ -9185,27 +9190,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="122" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="10" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B122" s="11" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="C122" s="11" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="D122" s="10" t="s">
         <v>85</v>
       </c>
       <c r="E122" s="11" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="F122" s="11" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="G122" s="11" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="H122" s="10" t="s">
         <v>21</v>
@@ -9214,13 +9219,13 @@
         <v>22</v>
       </c>
       <c r="J122" s="12" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="K122" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L122" s="14" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="M122" s="13" t="s">
         <v>26</v>
@@ -9229,27 +9234,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="123" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="10" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B123" s="11" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="C123" s="11" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="D123" s="10" t="s">
         <v>85</v>
       </c>
       <c r="E123" s="11" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="F123" s="11" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="G123" s="11" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="H123" s="10" t="s">
         <v>21</v>
@@ -9264,7 +9269,7 @@
         <v>247</v>
       </c>
       <c r="L123" s="14" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="M123" s="13" t="s">
         <v>26</v>
@@ -9273,27 +9278,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="124" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="10" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B124" s="11" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="C124" s="11" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="D124" s="10" t="s">
         <v>85</v>
       </c>
       <c r="E124" s="11" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="F124" s="11" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="G124" s="11" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="H124" s="10" t="s">
         <v>38</v>
@@ -9308,7 +9313,7 @@
         <v>24</v>
       </c>
       <c r="L124" s="14" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="M124" s="13" t="s">
         <v>26</v>
@@ -9317,27 +9322,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="125" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="10" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B125" s="11" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="C125" s="11" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="D125" s="10" t="s">
         <v>383</v>
       </c>
       <c r="E125" s="11" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="F125" s="11" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="G125" s="11" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="H125" s="10" t="s">
         <v>21</v>
@@ -9346,13 +9351,13 @@
         <v>22</v>
       </c>
       <c r="J125" s="12" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="K125" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L125" s="14" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="M125" s="13" t="s">
         <v>26</v>
@@ -9361,27 +9366,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="126" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="10" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="B126" s="11" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="C126" s="11" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="D126" s="10" t="s">
         <v>85</v>
       </c>
       <c r="E126" s="11" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="F126" s="11" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="G126" s="11" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="H126" s="10" t="s">
         <v>21</v>
@@ -9390,13 +9395,13 @@
         <v>22</v>
       </c>
       <c r="J126" s="12" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="K126" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L126" s="14" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="M126" s="13" t="s">
         <v>26</v>
@@ -9405,27 +9410,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="127" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="10" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="B127" s="11" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="C127" s="11" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="D127" s="10" t="s">
         <v>196</v>
       </c>
       <c r="E127" s="11" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="F127" s="11" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="G127" s="11" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="H127" s="10" t="s">
         <v>21</v>
@@ -9434,13 +9439,13 @@
         <v>22</v>
       </c>
       <c r="J127" s="12" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="K127" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L127" s="14" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="M127" s="13" t="s">
         <v>26</v>
@@ -9449,27 +9454,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="128" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="10" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="B128" s="11" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="C128" s="11" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="D128" s="10" t="s">
         <v>85</v>
       </c>
       <c r="E128" s="11" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="F128" s="11" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="G128" s="11" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="H128" s="10" t="s">
         <v>38</v>
@@ -9478,13 +9483,13 @@
         <v>22</v>
       </c>
       <c r="J128" s="12" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="K128" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L128" s="14" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="M128" s="13" t="s">
         <v>26</v>
@@ -9493,27 +9498,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="129" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="10" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="B129" s="11" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="C129" s="11" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="D129" s="10" t="s">
         <v>119</v>
       </c>
       <c r="E129" s="11" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="F129" s="11" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="G129" s="11" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="H129" s="10" t="s">
         <v>38</v>
@@ -9522,13 +9527,13 @@
         <v>22</v>
       </c>
       <c r="J129" s="12" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="K129" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L129" s="14" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="M129" s="13" t="s">
         <v>26</v>
@@ -9537,27 +9542,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="130" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="10" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="B130" s="11" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="C130" s="11" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="D130" s="10" t="s">
         <v>85</v>
       </c>
       <c r="E130" s="11" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="F130" s="11" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="G130" s="11" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="H130" s="10" t="s">
         <v>38</v>
@@ -9572,7 +9577,7 @@
         <v>24</v>
       </c>
       <c r="L130" s="14" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="M130" s="13" t="s">
         <v>26</v>
@@ -9581,27 +9586,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="131" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="10" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="B131" s="11" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="C131" s="11" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="D131" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E131" s="11" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F131" s="11" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="G131" s="11" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="H131" s="10" t="s">
         <v>21</v>
@@ -9616,7 +9621,7 @@
         <v>24</v>
       </c>
       <c r="L131" s="14" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="M131" s="13" t="s">
         <v>26</v>
@@ -9625,15 +9630,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="132" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="10" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="B132" s="11" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="C132" s="11" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="D132" s="10" t="s">
         <v>17</v>
@@ -9642,10 +9647,10 @@
         <v>29</v>
       </c>
       <c r="F132" s="11" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="G132" s="11" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="H132" s="10" t="s">
         <v>38</v>
@@ -9660,7 +9665,7 @@
         <v>24</v>
       </c>
       <c r="L132" s="14" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="M132" s="13" t="s">
         <v>26</v>
@@ -9669,27 +9674,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="133" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="10" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="B133" s="11" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="C133" s="11" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="D133" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E133" s="11" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="F133" s="11" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="G133" s="11" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="H133" s="10" t="s">
         <v>38</v>
@@ -9704,7 +9709,7 @@
         <v>247</v>
       </c>
       <c r="L133" s="14" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="M133" s="13" t="s">
         <v>26</v>
@@ -9713,15 +9718,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="134" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="10" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="B134" s="11" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="C134" s="11" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="D134" s="10" t="s">
         <v>85</v>
@@ -9730,10 +9735,10 @@
         <v>29</v>
       </c>
       <c r="F134" s="11" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="G134" s="11" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="H134" s="10" t="s">
         <v>80</v>
@@ -9757,27 +9762,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="135" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="10" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="B135" s="11" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="C135" s="11" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="D135" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E135" s="11" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
       <c r="F135" s="11" t="s">
-        <v>819</v>
+        <v>820</v>
       </c>
       <c r="G135" s="11" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="H135" s="10" t="s">
         <v>38</v>
@@ -9792,7 +9797,7 @@
         <v>24</v>
       </c>
       <c r="L135" s="14" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="M135" s="13" t="s">
         <v>26</v>
@@ -9801,27 +9806,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="136" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="10" t="s">
-        <v>822</v>
+        <v>823</v>
       </c>
       <c r="B136" s="11" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="C136" s="11" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="D136" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E136" s="11" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="F136" s="11" t="s">
-        <v>824</v>
+        <v>825</v>
       </c>
       <c r="G136" s="11" t="s">
-        <v>825</v>
+        <v>826</v>
       </c>
       <c r="H136" s="10" t="s">
         <v>38</v>
@@ -9836,7 +9841,7 @@
         <v>24</v>
       </c>
       <c r="L136" s="14" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="M136" s="13" t="s">
         <v>26</v>
@@ -9845,27 +9850,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="137" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="10" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="B137" s="11" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="C137" s="11" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="D137" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E137" s="11" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="F137" s="11" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="G137" s="11" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="H137" s="10" t="s">
         <v>80</v>
@@ -9880,7 +9885,7 @@
         <v>247</v>
       </c>
       <c r="L137" s="14" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="M137" s="13" t="s">
         <v>26</v>
@@ -9889,27 +9894,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="138" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="10" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="B138" s="11" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="C138" s="11" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="D138" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E138" s="11" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="F138" s="11" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="G138" s="11" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="H138" s="10" t="s">
         <v>38</v>
@@ -9924,7 +9929,7 @@
         <v>24</v>
       </c>
       <c r="L138" s="14" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="M138" s="13" t="s">
         <v>26</v>
@@ -9933,27 +9938,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="139" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="10" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="B139" s="11" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="C139" s="11" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="D139" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E139" s="11" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="F139" s="11" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="G139" s="11" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="H139" s="10" t="s">
         <v>38</v>
@@ -9977,27 +9982,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="140" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="10" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="B140" s="11" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="C140" s="11" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="D140" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E140" s="11" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="F140" s="11" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="G140" s="11" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="H140" s="10" t="s">
         <v>38</v>
@@ -10012,7 +10017,7 @@
         <v>24</v>
       </c>
       <c r="L140" s="14" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="M140" s="13" t="s">
         <v>26</v>
@@ -10021,15 +10026,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="141" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="10" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="B141" s="11" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="C141" s="11" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="D141" s="10" t="s">
         <v>17</v>
@@ -10038,10 +10043,10 @@
         <v>29</v>
       </c>
       <c r="F141" s="11" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="G141" s="11" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="H141" s="10" t="s">
         <v>80</v>
@@ -10065,15 +10070,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="142" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="10" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="B142" s="11" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="C142" s="11" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="D142" s="10" t="s">
         <v>17</v>
@@ -10082,10 +10087,10 @@
         <v>29</v>
       </c>
       <c r="F142" s="11" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="G142" s="11" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="H142" s="10" t="s">
         <v>21</v>
@@ -10094,7 +10099,7 @@
         <v>22</v>
       </c>
       <c r="J142" s="12" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="K142" s="13" t="s">
         <v>24</v>
@@ -10109,15 +10114,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="143" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="10" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="B143" s="11" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="C143" s="11" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="D143" s="10" t="s">
         <v>119</v>
@@ -10126,10 +10131,10 @@
         <v>29</v>
       </c>
       <c r="F143" s="11" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="G143" s="11" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="H143" s="10" t="s">
         <v>21</v>
@@ -10138,7 +10143,7 @@
         <v>22</v>
       </c>
       <c r="J143" s="12" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="K143" s="13" t="s">
         <v>24</v>
@@ -10153,15 +10158,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="144" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="10" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="B144" s="11" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="C144" s="11" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="D144" s="10" t="s">
         <v>17</v>
@@ -10170,10 +10175,10 @@
         <v>29</v>
       </c>
       <c r="F144" s="11" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="G144" s="11" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="H144" s="10" t="s">
         <v>21</v>
@@ -10182,13 +10187,13 @@
         <v>22</v>
       </c>
       <c r="J144" s="12" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="K144" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L144" s="14" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="M144" s="13" t="s">
         <v>26</v>
@@ -10197,15 +10202,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="145" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="10" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="B145" s="11" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="C145" s="11" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="D145" s="10" t="s">
         <v>17</v>
@@ -10214,10 +10219,10 @@
         <v>29</v>
       </c>
       <c r="F145" s="11" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="G145" s="11" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="H145" s="10" t="s">
         <v>38</v>
@@ -10226,13 +10231,13 @@
         <v>22</v>
       </c>
       <c r="J145" s="12" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="K145" s="13" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="L145" s="14" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="M145" s="13" t="s">
         <v>26</v>
@@ -10241,27 +10246,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="146" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="10" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="B146" s="11" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="C146" s="11" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="D146" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E146" s="11" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="F146" s="11" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="G146" s="11" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="H146" s="10" t="s">
         <v>38</v>
@@ -10270,7 +10275,7 @@
         <v>22</v>
       </c>
       <c r="J146" s="12" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="K146" s="13" t="s">
         <v>24</v>
@@ -10285,27 +10290,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="147" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="10" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="B147" s="11" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="C147" s="11" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="D147" s="10" t="s">
         <v>119</v>
       </c>
       <c r="E147" s="11" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="F147" s="11" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="G147" s="11" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
       <c r="H147" s="10" t="s">
         <v>21</v>
@@ -10314,13 +10319,13 @@
         <v>22</v>
       </c>
       <c r="J147" s="12" t="s">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="K147" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L147" s="14" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="M147" s="13" t="s">
         <v>26</v>
@@ -10329,27 +10334,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="148" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="10" t="s">
-        <v>892</v>
+        <v>893</v>
       </c>
       <c r="B148" s="11" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="C148" s="11" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
       <c r="D148" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E148" s="11" t="s">
-        <v>894</v>
+        <v>895</v>
       </c>
       <c r="F148" s="11" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
       <c r="G148" s="11" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="H148" s="10" t="s">
         <v>21</v>
@@ -10358,13 +10363,13 @@
         <v>22</v>
       </c>
       <c r="J148" s="12" t="s">
-        <v>897</v>
+        <v>898</v>
       </c>
       <c r="K148" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L148" s="14" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
       <c r="M148" s="13" t="s">
         <v>26</v>
@@ -10373,15 +10378,15 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="149" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="10" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="B149" s="11" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="C149" s="11" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
       <c r="D149" s="10" t="s">
         <v>119</v>
@@ -10390,10 +10395,10 @@
         <v>29</v>
       </c>
       <c r="F149" s="11" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="G149" s="11" t="s">
-        <v>902</v>
+        <v>903</v>
       </c>
       <c r="H149" s="10" t="s">
         <v>21</v>
@@ -10402,13 +10407,13 @@
         <v>22</v>
       </c>
       <c r="J149" s="12" t="s">
-        <v>903</v>
+        <v>904</v>
       </c>
       <c r="K149" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L149" s="14" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="M149" s="13" t="s">
         <v>26</v>
@@ -10417,27 +10422,27 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="150" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="10" t="s">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="B150" s="11" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="C150" s="11" t="s">
-        <v>906</v>
+        <v>907</v>
       </c>
       <c r="D150" s="10" t="s">
         <v>383</v>
       </c>
       <c r="E150" s="11" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="F150" s="11" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="G150" s="11" t="s">
-        <v>909</v>
+        <v>910</v>
       </c>
       <c r="H150" s="10" t="s">
         <v>21</v>
@@ -10446,13 +10451,13 @@
         <v>22</v>
       </c>
       <c r="J150" s="12" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="K150" s="13" t="s">
         <v>24</v>
       </c>
       <c r="L150" s="14" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="M150" s="13" t="s">
         <v>26</v>
@@ -10500,14 +10505,14 @@
     <col min="8" max="9" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -10515,28 +10520,28 @@
         <v>1</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="C4" s="18" t="s">
         <v>24</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="E4" s="18" t="s">
         <v>247</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
       <c r="G4" s="18" t="s">
         <v>8</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>976</v>
+        <v>977</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -10837,7 +10842,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B13" s="20">
         <f>COUNTIF('حالات الاختبار'!$B$2:$B$150,A13)</f>
@@ -10874,7 +10879,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="B14" s="20">
         <f>COUNTIF('حالات الاختبار'!$B$2:$B$150,A14)</f>
@@ -10911,7 +10916,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="B15" s="20">
         <f>COUNTIF('حالات الاختبار'!$B$2:$B$150,A15)</f>
@@ -10948,7 +10953,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="B16" s="20">
         <f>COUNTIF('حالات الاختبار'!$B$2:$B$150,A16)</f>
@@ -10985,7 +10990,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="B17" s="20">
         <f>COUNTIF('حالات الاختبار'!$B$2:$B$150,A17)</f>
@@ -11022,7 +11027,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B18" s="20">
         <f>COUNTIF('حالات الاختبار'!$B$2:$B$150,A18)</f>
@@ -11059,7 +11064,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B19" s="20">
         <f>COUNTIF('حالات الاختبار'!$B$2:$B$150,A19)</f>
@@ -11096,7 +11101,7 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B20" s="20">
         <f>COUNTIF('حالات الاختبار'!$B$2:$B$150,A20)</f>
@@ -11133,7 +11138,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="B21" s="20">
         <f>COUNTIF('حالات الاختبار'!$B$2:$B$150,A21)</f>
@@ -11170,7 +11175,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="19" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="B22" s="20">
         <f>COUNTIF('حالات الاختبار'!$B$2:$B$150,A22)</f>
@@ -11207,7 +11212,7 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="B23" s="20">
         <f>COUNTIF('حالات الاختبار'!$B$2:$B$150,A23)</f>
@@ -11244,7 +11249,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="B24" s="20">
         <f>COUNTIF('حالات الاختبار'!$B$2:$B$150,A24)</f>
@@ -11281,7 +11286,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="22" t="s">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="B25" s="23">
         <f t="shared" ref="B25:G25" si="3">SUM(B5:B24)</f>
@@ -11316,9 +11321,9 @@
         <v>0.99310344827586206</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>978</v>
+        <v>979</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -11326,16 +11331,16 @@
         <v>7</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="C29" s="18" t="s">
         <v>24</v>
       </c>
       <c r="D29" s="18" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -11403,7 +11408,7 @@
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="25" t="s">
-        <v>979</v>
+        <v>980</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Brand: the store logo and its colors
- Palette from the logo: navy #073060 (brand) and orange #f4750d (accent);
  cooler neutrals. New «accent» button for the main actions: بيع جديد,
  الدفع, اعتماد الفاتورة.
- App, home-screen and browser icons from the logo's mark (house + «قويدر»),
  readable at small sizes; the mark in the header and sidebar; the full logo
  on a light sign-in page. theme_color/background_color updated.
- Original artwork kept in docs/brand/logo-original.png.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Qwader-Test-Cases.xlsx
+++ b/docs/Qwader-Test-Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Qwader\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53AE89D1-EC99-403D-BBD9-180DCAD33118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{436A5771-0DAF-4366-9FEC-8BDB66CC0579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2617,7 +2617,7 @@
     <t>1. الحساب الشخصي ← تثبيت التطبيق</t>
   </si>
   <si>
-    <t>تظهر أيقونة «معرض قويدر» (البيت وحرف ق) على الشاشة</t>
+    <t>تظهر أيقونة «معرض قويدر» (شعار البيت وكلمة «قويدر» بالكحلي والبرتقالي) على الشاشة</t>
   </si>
   <si>
     <t>قابل للتثبيت: «معرض قويدر للأدوات والأجهزة المنزلية»، 4 أيقونات (التثبيت الفعلي يُجرَّب على الجوال)</t>
@@ -3741,7 +3741,7 @@
         <v>951</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>952</v>
       </c>
@@ -3973,7 +3973,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>14</v>
       </c>
@@ -4017,7 +4017,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>27</v>
       </c>
@@ -4061,7 +4061,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>33</v>
       </c>
@@ -4105,7 +4105,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>41</v>
       </c>
@@ -4149,7 +4149,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>47</v>
       </c>
@@ -4193,7 +4193,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>53</v>
       </c>
@@ -4237,7 +4237,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>59</v>
       </c>
@@ -4281,7 +4281,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>65</v>
       </c>
@@ -4325,7 +4325,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
         <v>70</v>
       </c>
@@ -4369,7 +4369,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>76</v>
       </c>
@@ -4413,7 +4413,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
         <v>82</v>
       </c>
@@ -4457,7 +4457,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>88</v>
       </c>
@@ -4501,7 +4501,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
         <v>94</v>
       </c>
@@ -4545,7 +4545,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>100</v>
       </c>
@@ -4589,7 +4589,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
         <v>105</v>
       </c>
@@ -4633,7 +4633,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
         <v>111</v>
       </c>
@@ -4677,7 +4677,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
         <v>117</v>
       </c>
@@ -4721,7 +4721,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
         <v>123</v>
       </c>
@@ -4765,7 +4765,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
         <v>128</v>
       </c>
@@ -4809,7 +4809,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
         <v>133</v>
       </c>
@@ -4853,7 +4853,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
         <v>138</v>
       </c>
@@ -4897,7 +4897,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
         <v>144</v>
       </c>
@@ -4941,7 +4941,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
         <v>151</v>
       </c>
@@ -4985,7 +4985,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
         <v>158</v>
       </c>
@@ -5029,7 +5029,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
         <v>164</v>
       </c>
@@ -5073,7 +5073,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
         <v>169</v>
       </c>
@@ -5117,7 +5117,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
         <v>175</v>
       </c>
@@ -5161,7 +5161,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
         <v>180</v>
       </c>
@@ -5205,7 +5205,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
         <v>187</v>
       </c>
@@ -5249,7 +5249,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
         <v>193</v>
       </c>
@@ -5293,7 +5293,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
         <v>200</v>
       </c>
@@ -5337,7 +5337,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
         <v>205</v>
       </c>
@@ -5381,7 +5381,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
         <v>210</v>
       </c>
@@ -5425,7 +5425,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
         <v>215</v>
       </c>
@@ -5469,7 +5469,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
         <v>223</v>
       </c>
@@ -5513,7 +5513,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
         <v>228</v>
       </c>
@@ -5557,7 +5557,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="38" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
         <v>235</v>
       </c>
@@ -5601,7 +5601,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="39" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
         <v>242</v>
       </c>
@@ -5645,7 +5645,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="40" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
         <v>249</v>
       </c>
@@ -5689,7 +5689,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="41" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
         <v>256</v>
       </c>
@@ -5733,7 +5733,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
         <v>262</v>
       </c>
@@ -5777,7 +5777,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="43" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
         <v>269</v>
       </c>
@@ -5821,7 +5821,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="44" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
         <v>276</v>
       </c>
@@ -5865,7 +5865,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="45" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
         <v>282</v>
       </c>
@@ -5909,7 +5909,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="46" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
         <v>286</v>
       </c>
@@ -5953,7 +5953,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
         <v>292</v>
       </c>
@@ -5997,7 +5997,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="48" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
         <v>299</v>
       </c>
@@ -6041,7 +6041,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="49" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
         <v>305</v>
       </c>
@@ -6085,7 +6085,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="50" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
         <v>311</v>
       </c>
@@ -6129,7 +6129,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="51" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
         <v>318</v>
       </c>
@@ -6173,7 +6173,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="52" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
         <v>325</v>
       </c>
@@ -6217,7 +6217,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="53" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
         <v>332</v>
       </c>
@@ -6261,7 +6261,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="54" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
         <v>337</v>
       </c>
@@ -6305,7 +6305,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="55" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
         <v>343</v>
       </c>
@@ -6349,7 +6349,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="56" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
         <v>348</v>
       </c>
@@ -6393,7 +6393,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
         <v>355</v>
       </c>
@@ -6437,7 +6437,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
         <v>362</v>
       </c>
@@ -6481,7 +6481,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="59" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
         <v>368</v>
       </c>
@@ -6525,7 +6525,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="60" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
         <v>375</v>
       </c>
@@ -6569,7 +6569,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="61" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
         <v>381</v>
       </c>
@@ -6613,7 +6613,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
         <v>389</v>
       </c>
@@ -6657,7 +6657,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
         <v>396</v>
       </c>
@@ -6701,7 +6701,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="64" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
         <v>402</v>
       </c>
@@ -6745,7 +6745,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="65" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
         <v>406</v>
       </c>
@@ -6789,7 +6789,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="66" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
         <v>412</v>
       </c>
@@ -6833,7 +6833,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="67" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
         <v>419</v>
       </c>
@@ -6877,7 +6877,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="68" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
         <v>425</v>
       </c>
@@ -6921,7 +6921,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="69" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
         <v>431</v>
       </c>
@@ -6965,7 +6965,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="70" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
         <v>436</v>
       </c>
@@ -7009,7 +7009,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="71" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
         <v>442</v>
       </c>
@@ -7053,7 +7053,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="72" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
         <v>447</v>
       </c>
@@ -7097,7 +7097,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="73" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
         <v>453</v>
       </c>
@@ -7141,7 +7141,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="74" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
         <v>459</v>
       </c>
@@ -7185,7 +7185,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="75" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="10" t="s">
         <v>466</v>
       </c>
@@ -7229,7 +7229,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="76" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="10" t="s">
         <v>471</v>
       </c>
@@ -7273,7 +7273,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="77" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="10" t="s">
         <v>477</v>
       </c>
@@ -7317,7 +7317,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="78" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="10" t="s">
         <v>482</v>
       </c>
@@ -7361,7 +7361,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="79" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="10" t="s">
         <v>488</v>
       </c>
@@ -7405,7 +7405,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="80" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="10" t="s">
         <v>493</v>
       </c>
@@ -7449,7 +7449,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="81" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="10" t="s">
         <v>499</v>
       </c>
@@ -7493,7 +7493,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="82" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="10" t="s">
         <v>505</v>
       </c>
@@ -7537,7 +7537,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="83" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="10" t="s">
         <v>512</v>
       </c>
@@ -7581,7 +7581,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="84" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="10" t="s">
         <v>518</v>
       </c>
@@ -7625,7 +7625,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="85" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="10" t="s">
         <v>523</v>
       </c>
@@ -7669,7 +7669,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="86" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="10" t="s">
         <v>530</v>
       </c>
@@ -7713,7 +7713,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="87" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="10" t="s">
         <v>536</v>
       </c>
@@ -7757,7 +7757,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="88" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="10" t="s">
         <v>541</v>
       </c>
@@ -7801,7 +7801,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="89" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="10" t="s">
         <v>549</v>
       </c>
@@ -7845,7 +7845,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="90" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="10" t="s">
         <v>555</v>
       </c>
@@ -7889,7 +7889,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="91" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="10" t="s">
         <v>560</v>
       </c>
@@ -7933,7 +7933,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="92" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="10" t="s">
         <v>567</v>
       </c>
@@ -7977,7 +7977,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="93" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="10" t="s">
         <v>572</v>
       </c>
@@ -8021,7 +8021,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="94" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="10" t="s">
         <v>578</v>
       </c>
@@ -8065,7 +8065,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="95" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="10" t="s">
         <v>585</v>
       </c>
@@ -8109,7 +8109,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="96" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="10" t="s">
         <v>590</v>
       </c>
@@ -8153,7 +8153,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="97" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="10" t="s">
         <v>597</v>
       </c>
@@ -8197,7 +8197,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="98" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="10" t="s">
         <v>603</v>
       </c>
@@ -8241,7 +8241,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="99" spans="1:14" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:14" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="10" t="s">
         <v>608</v>
       </c>
@@ -8285,7 +8285,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="100" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="10" t="s">
         <v>615</v>
       </c>
@@ -8329,7 +8329,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="101" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="10" t="s">
         <v>621</v>
       </c>
@@ -8373,7 +8373,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="102" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="10" t="s">
         <v>628</v>
       </c>
@@ -8417,7 +8417,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="103" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="10" t="s">
         <v>633</v>
       </c>
@@ -8461,7 +8461,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="104" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="10" t="s">
         <v>640</v>
       </c>
@@ -8505,7 +8505,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="105" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="10" t="s">
         <v>645</v>
       </c>
@@ -8549,7 +8549,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="106" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="10" t="s">
         <v>651</v>
       </c>
@@ -8593,7 +8593,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="107" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="10" t="s">
         <v>657</v>
       </c>
@@ -8637,7 +8637,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="108" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="10" t="s">
         <v>664</v>
       </c>
@@ -8681,7 +8681,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="109" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="10" t="s">
         <v>672</v>
       </c>
@@ -8725,7 +8725,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="110" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="10" t="s">
         <v>677</v>
       </c>
@@ -8769,7 +8769,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="111" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="10" t="s">
         <v>684</v>
       </c>
@@ -8813,7 +8813,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="112" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="10" t="s">
         <v>689</v>
       </c>
@@ -8857,7 +8857,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="113" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="10" t="s">
         <v>694</v>
       </c>
@@ -8901,7 +8901,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="114" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="10" t="s">
         <v>700</v>
       </c>
@@ -8945,7 +8945,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="115" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="10" t="s">
         <v>707</v>
       </c>
@@ -8989,7 +8989,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="116" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="10" t="s">
         <v>714</v>
       </c>
@@ -9033,7 +9033,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="117" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="10" t="s">
         <v>719</v>
       </c>
@@ -9077,7 +9077,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="118" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="10" t="s">
         <v>725</v>
       </c>
@@ -9121,7 +9121,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="119" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="10" t="s">
         <v>730</v>
       </c>
@@ -9165,7 +9165,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="120" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="10" t="s">
         <v>734</v>
       </c>
@@ -9209,7 +9209,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="121" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="10" t="s">
         <v>741</v>
       </c>
@@ -9253,7 +9253,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="122" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="10" t="s">
         <v>746</v>
       </c>
@@ -9297,7 +9297,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="123" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="10" t="s">
         <v>753</v>
       </c>
@@ -9341,7 +9341,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="124" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="10" t="s">
         <v>758</v>
       </c>
@@ -9385,7 +9385,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="125" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="10" t="s">
         <v>764</v>
       </c>
@@ -9429,7 +9429,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="126" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="10" t="s">
         <v>772</v>
       </c>
@@ -9473,7 +9473,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="127" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="10" t="s">
         <v>778</v>
       </c>
@@ -9517,7 +9517,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="128" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="10" t="s">
         <v>784</v>
       </c>
@@ -9561,7 +9561,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="129" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="10" t="s">
         <v>791</v>
       </c>
@@ -9605,7 +9605,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="130" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="10" t="s">
         <v>796</v>
       </c>
@@ -9649,7 +9649,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="131" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="10" t="s">
         <v>801</v>
       </c>
@@ -9693,7 +9693,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="132" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="10" t="s">
         <v>806</v>
       </c>
@@ -9737,7 +9737,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="133" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="10" t="s">
         <v>811</v>
       </c>
@@ -9781,7 +9781,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="134" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="10" t="s">
         <v>816</v>
       </c>
@@ -9825,7 +9825,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="135" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="10" t="s">
         <v>822</v>
       </c>
@@ -9869,7 +9869,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="136" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="10" t="s">
         <v>827</v>
       </c>
@@ -9913,7 +9913,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="137" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="10" t="s">
         <v>833</v>
       </c>
@@ -9957,7 +9957,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="138" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="10" t="s">
         <v>837</v>
       </c>
@@ -10001,7 +10001,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="139" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="10" t="s">
         <v>844</v>
       </c>
@@ -10045,7 +10045,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="140" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="10" t="s">
         <v>849</v>
       </c>
@@ -10089,7 +10089,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="141" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="10" t="s">
         <v>855</v>
       </c>
@@ -10133,7 +10133,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="142" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="10" t="s">
         <v>861</v>
       </c>
@@ -10177,7 +10177,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="143" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="10" t="s">
         <v>866</v>
       </c>
@@ -10221,7 +10221,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="144" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="10" t="s">
         <v>872</v>
       </c>
@@ -10265,7 +10265,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="145" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="10" t="s">
         <v>876</v>
       </c>
@@ -10309,7 +10309,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="146" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="10" t="s">
         <v>882</v>
       </c>
@@ -10353,7 +10353,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="147" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="10" t="s">
         <v>887</v>
       </c>
@@ -10397,7 +10397,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="148" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="10" t="s">
         <v>893</v>
       </c>
@@ -10441,7 +10441,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="149" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="10" t="s">
         <v>899</v>
       </c>
@@ -10485,7 +10485,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="150" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="10" t="s">
         <v>905</v>
       </c>
@@ -10529,7 +10529,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="151" spans="1:14" ht="51" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="10" t="s">
         <v>913</v>
       </c>
@@ -10573,7 +10573,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="152" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="10" t="s">
         <v>920</v>
       </c>
@@ -10617,7 +10617,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="153" spans="1:14" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="10" t="s">
         <v>926</v>
       </c>
@@ -10700,7 +10700,7 @@
     <col min="8" max="9" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
         <v>993</v>
       </c>
@@ -11516,7 +11516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>1000</v>
       </c>

</xml_diff>

<commit_message>
Damaged and lost stock lowers the capital in goods, not expenses or profit
The store's rule: المصروفات = salaries, repairs and running costs only;
صافي الربح = إجمالي الربح − المصروفات. Stock damaged/lost or counted over is
shown in a new «رأس المال في البضاعة» section with the stock value, and in the
Excel export next to it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Qwader-Test-Cases.xlsx
+++ b/docs/Qwader-Test-Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Qwader\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{436A5771-0DAF-4366-9FEC-8BDB66CC0579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB49C84F-EAE2-43CB-BF58-A7EA2BD69198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1018,7 +1018,7 @@
     <t>1. المخزون ← تعديل ← تالف 1</t>
   </si>
   <si>
-    <t>الكمية 4 وتظهر كخسارة في التقارير</t>
+    <t>الكمية 4، وتظهر في التقارير تحت «رأس المال في البضاعة» لا في المصروفات</t>
   </si>
   <si>
     <t>Weighted_average_follows_purchases_shrinkage_and_purchase_returns</t>
@@ -2217,7 +2217,7 @@
     <t>1. التقارير ← اليوم</t>
   </si>
   <si>
-    <t>المبيعات (الإيرادات) = المبيعات − الخصومات − المرتجعات؛ إجمالي الربح = المبيعات − سعر الشراء؛ المصروفات = رواتب وأعطال ومصاريف تشغيلية + التالف؛ صافي الربح = إجمالي الربح − المصروفات</t>
+    <t>المبيعات (الإيرادات) = المبيعات − الخصومات − المرتجعات؛ إجمالي الربح = المبيعات − سعر الشراء؛ المصروفات = رواتب وأعطال ومصاريف تشغيلية فقط؛ صافي الربح = إجمالي الربح − المصروفات؛ التالف والمفقود يُنقص قيمة المخزون (رأس المال) ولا يدخل في الربح</t>
   </si>
   <si>
     <t>Profit_and_loss_follows_the_accounting_rules</t>

</xml_diff>